<commit_message>
Refactor weight handling methods in DenseLayer and NeuralNetwork
</commit_message>
<xml_diff>
--- a/full/sliding_window_results_window_1.xlsx
+++ b/full/sliding_window_results_window_1.xlsx
@@ -463,13 +463,13 @@
         <v>28.98</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>29.72175776911019</v>
       </c>
       <c r="D2" t="n">
-        <v>-28.98</v>
+        <v>0.7417577691101904</v>
       </c>
       <c r="E2" t="n">
-        <v>839.8404</v>
+        <v>0.5502045880353266</v>
       </c>
     </row>
     <row r="3">
@@ -480,13 +480,13 @@
         <v>29.15</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>30.02891384579398</v>
       </c>
       <c r="D3" t="n">
-        <v>-29.15</v>
+        <v>0.8789138457939778</v>
       </c>
       <c r="E3" t="n">
-        <v>849.7225</v>
+        <v>0.7724895483283601</v>
       </c>
     </row>
     <row r="4">
@@ -497,13 +497,13 @@
         <v>29.35</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>29.87532757460375</v>
       </c>
       <c r="D4" t="n">
-        <v>-29.35</v>
+        <v>0.5253275746037467</v>
       </c>
       <c r="E4" t="n">
-        <v>861.4225000000001</v>
+        <v>0.275969060639055</v>
       </c>
     </row>
     <row r="5">
@@ -514,13 +514,13 @@
         <v>29.37</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>29.64943781981881</v>
       </c>
       <c r="D5" t="n">
-        <v>-29.37</v>
+        <v>0.2794378198188099</v>
       </c>
       <c r="E5" t="n">
-        <v>862.5969</v>
+        <v>0.07808549514508965</v>
       </c>
     </row>
     <row r="6">
@@ -531,13 +531,13 @@
         <v>29.54</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>30.2197193266033</v>
       </c>
       <c r="D6" t="n">
-        <v>-29.54</v>
+        <v>0.6797193266032977</v>
       </c>
       <c r="E6" t="n">
-        <v>872.6116</v>
+        <v>0.4620183629580405</v>
       </c>
     </row>
     <row r="7">
@@ -548,13 +548,13 @@
         <v>29.55</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>30.16524852836157</v>
       </c>
       <c r="D7" t="n">
-        <v>-29.55</v>
+        <v>0.6152485283615654</v>
       </c>
       <c r="E7" t="n">
-        <v>873.2025</v>
+        <v>0.378530751651072</v>
       </c>
     </row>
     <row r="8">
@@ -565,13 +565,13 @@
         <v>29.75</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>30.95421275670812</v>
       </c>
       <c r="D8" t="n">
-        <v>-29.75</v>
+        <v>1.20421275670812</v>
       </c>
       <c r="E8" t="n">
-        <v>885.0625</v>
+        <v>1.45012836341857</v>
       </c>
     </row>
     <row r="9">
@@ -582,13 +582,13 @@
         <v>29.84</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>30.3238393500008</v>
       </c>
       <c r="D9" t="n">
-        <v>-29.84</v>
+        <v>0.483839350000796</v>
       </c>
       <c r="E9" t="n">
-        <v>890.4256</v>
+        <v>0.2341005166091928</v>
       </c>
     </row>
     <row r="10">
@@ -599,13 +599,13 @@
         <v>29.81</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>29.46879379716013</v>
       </c>
       <c r="D10" t="n">
-        <v>-29.81</v>
+        <v>-0.3412062028398708</v>
       </c>
       <c r="E10" t="n">
-        <v>888.6360999999999</v>
+        <v>0.116421672856403</v>
       </c>
     </row>
     <row r="11">
@@ -616,13 +616,13 @@
         <v>29.92</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>30.68162427992516</v>
       </c>
       <c r="D11" t="n">
-        <v>-29.92</v>
+        <v>0.761624279925158</v>
       </c>
       <c r="E11" t="n">
-        <v>895.2064000000001</v>
+        <v>0.5800715437715155</v>
       </c>
     </row>
     <row r="12">
@@ -633,13 +633,13 @@
         <v>29.98</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>30.02526259058906</v>
       </c>
       <c r="D12" t="n">
-        <v>-29.98</v>
+        <v>0.04526259058906135</v>
       </c>
       <c r="E12" t="n">
-        <v>898.8004000000001</v>
+        <v>0.002048702106832985</v>
       </c>
     </row>
     <row r="13">
@@ -650,13 +650,13 @@
         <v>30.04</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>29.65885848788355</v>
       </c>
       <c r="D13" t="n">
-        <v>-30.04</v>
+        <v>-0.3811415121164501</v>
       </c>
       <c r="E13" t="n">
-        <v>902.4015999999999</v>
+        <v>0.1452688522584141</v>
       </c>
     </row>
     <row r="14">
@@ -667,13 +667,13 @@
         <v>30.21</v>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>30.0738608790388</v>
       </c>
       <c r="D14" t="n">
-        <v>-30.21</v>
+        <v>-0.1361391209612037</v>
       </c>
       <c r="E14" t="n">
-        <v>912.6441000000001</v>
+        <v>0.01853386025608926</v>
       </c>
     </row>
     <row r="15">
@@ -684,13 +684,13 @@
         <v>30.22</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>29.9260358867717</v>
       </c>
       <c r="D15" t="n">
-        <v>-30.22</v>
+        <v>-0.2939641132282951</v>
       </c>
       <c r="E15" t="n">
-        <v>913.2483999999999</v>
+        <v>0.08641489986609789</v>
       </c>
     </row>
     <row r="16">
@@ -701,13 +701,13 @@
         <v>30.38</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>29.94177716779699</v>
       </c>
       <c r="D16" t="n">
-        <v>-30.38</v>
+        <v>-0.4382228322030066</v>
       </c>
       <c r="E16" t="n">
-        <v>922.9444</v>
+        <v>0.1920392506640245</v>
       </c>
     </row>
     <row r="17">
@@ -718,13 +718,13 @@
         <v>30.44</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>29.90366860471718</v>
       </c>
       <c r="D17" t="n">
-        <v>-30.44</v>
+        <v>-0.5363313952828221</v>
       </c>
       <c r="E17" t="n">
-        <v>926.5936</v>
+        <v>0.2876513655660188</v>
       </c>
     </row>
     <row r="18">
@@ -735,13 +735,13 @@
         <v>30.48</v>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>29.86792644700605</v>
       </c>
       <c r="D18" t="n">
-        <v>-30.48</v>
+        <v>-0.6120735529939552</v>
       </c>
       <c r="E18" t="n">
-        <v>929.0304</v>
+        <v>0.374634034274644</v>
       </c>
     </row>
     <row r="19">
@@ -752,13 +752,13 @@
         <v>30.69</v>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>30.78666544642995</v>
       </c>
       <c r="D19" t="n">
-        <v>-30.69</v>
+        <v>0.09666544642994523</v>
       </c>
       <c r="E19" t="n">
-        <v>941.8761000000001</v>
+        <v>0.009344208533500611</v>
       </c>
     </row>
     <row r="20">
@@ -769,13 +769,13 @@
         <v>30.75</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>30.99431524769091</v>
       </c>
       <c r="D20" t="n">
-        <v>-30.75</v>
+        <v>0.2443152476909134</v>
       </c>
       <c r="E20" t="n">
-        <v>945.5625</v>
+        <v>0.05968994025427236</v>
       </c>
     </row>
     <row r="21">
@@ -786,13 +786,13 @@
         <v>30.94</v>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>31.60933116519394</v>
       </c>
       <c r="D21" t="n">
-        <v>-30.94</v>
+        <v>0.6693311651939347</v>
       </c>
       <c r="E21" t="n">
-        <v>957.2836000000001</v>
+        <v>0.4480042086998702</v>
       </c>
     </row>
     <row r="22">
@@ -803,13 +803,13 @@
         <v>30.95</v>
       </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v>31.35647702173609</v>
       </c>
       <c r="D22" t="n">
-        <v>-30.95</v>
+        <v>0.4064770217360909</v>
       </c>
       <c r="E22" t="n">
-        <v>957.9024999999999</v>
+        <v>0.1652235691994425</v>
       </c>
     </row>
     <row r="23">
@@ -820,13 +820,13 @@
         <v>31.02</v>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>31.14129646547685</v>
       </c>
       <c r="D23" t="n">
-        <v>-31.02</v>
+        <v>0.1212964654768527</v>
       </c>
       <c r="E23" t="n">
-        <v>962.2404</v>
+        <v>0.01471283253717732</v>
       </c>
     </row>
     <row r="24">
@@ -837,13 +837,13 @@
         <v>31.12</v>
       </c>
       <c r="C24" t="n">
-        <v>0</v>
+        <v>31.11198262567547</v>
       </c>
       <c r="D24" t="n">
-        <v>-31.12</v>
+        <v>-0.008017374324534643</v>
       </c>
       <c r="E24" t="n">
-        <v>968.4544000000001</v>
+        <v>6.427829105970732e-05</v>
       </c>
     </row>
     <row r="25">
@@ -854,13 +854,13 @@
         <v>31.28</v>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>31.61760285234385</v>
       </c>
       <c r="D25" t="n">
-        <v>-31.28</v>
+        <v>0.3376028523438528</v>
       </c>
       <c r="E25" t="n">
-        <v>978.4384000000001</v>
+        <v>0.1139756859107053</v>
       </c>
     </row>
     <row r="26">
@@ -871,13 +871,13 @@
         <v>31.38</v>
       </c>
       <c r="C26" t="n">
-        <v>0</v>
+        <v>31.5746255466973</v>
       </c>
       <c r="D26" t="n">
-        <v>-31.38</v>
+        <v>0.1946255466973028</v>
       </c>
       <c r="E26" t="n">
-        <v>984.7044</v>
+        <v>0.037879103427224</v>
       </c>
     </row>
     <row r="27">
@@ -888,13 +888,13 @@
         <v>31.58</v>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>31.46276909702048</v>
       </c>
       <c r="D27" t="n">
-        <v>-31.58</v>
+        <v>-0.117230902979518</v>
       </c>
       <c r="E27" t="n">
-        <v>997.2963999999999</v>
+        <v>0.01374308461339316</v>
       </c>
     </row>
     <row r="28">
@@ -905,13 +905,13 @@
         <v>31.65</v>
       </c>
       <c r="C28" t="n">
-        <v>0</v>
+        <v>31.6124046137601</v>
       </c>
       <c r="D28" t="n">
-        <v>-31.65</v>
+        <v>-0.03759538623989656</v>
       </c>
       <c r="E28" t="n">
-        <v>1001.7225</v>
+        <v>0.001413413066527003</v>
       </c>
     </row>
     <row r="29">
@@ -922,13 +922,13 @@
         <v>31.88</v>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>32.07227687734462</v>
       </c>
       <c r="D29" t="n">
-        <v>-31.88</v>
+        <v>0.1922768773446215</v>
       </c>
       <c r="E29" t="n">
-        <v>1016.3344</v>
+        <v>0.03697039756139862</v>
       </c>
     </row>
     <row r="30">
@@ -939,13 +939,13 @@
         <v>32.28</v>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>32.43597484441806</v>
       </c>
       <c r="D30" t="n">
-        <v>-32.28</v>
+        <v>0.1559748444180542</v>
       </c>
       <c r="E30" t="n">
-        <v>1041.9984</v>
+        <v>0.02432815209123622</v>
       </c>
     </row>
     <row r="31">
@@ -956,13 +956,13 @@
         <v>32.45</v>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
+        <v>32.75777595936748</v>
       </c>
       <c r="D31" t="n">
-        <v>-32.45</v>
+        <v>0.3077759593674756</v>
       </c>
       <c r="E31" t="n">
-        <v>1053.0025</v>
+        <v>0.09472604116456999</v>
       </c>
     </row>
     <row r="32">
@@ -973,13 +973,13 @@
         <v>32.85</v>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>34.12422113804068</v>
       </c>
       <c r="D32" t="n">
-        <v>-32.85</v>
+        <v>1.27422113804068</v>
       </c>
       <c r="E32" t="n">
-        <v>1079.1225</v>
+        <v>1.623639508629686</v>
       </c>
     </row>
     <row r="33">
@@ -990,13 +990,13 @@
         <v>32.9</v>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>33.96927027946951</v>
       </c>
       <c r="D33" t="n">
-        <v>-32.9</v>
+        <v>1.069270279469514</v>
       </c>
       <c r="E33" t="n">
-        <v>1082.41</v>
+        <v>1.143338930556812</v>
       </c>
     </row>
     <row r="34">
@@ -1007,13 +1007,13 @@
         <v>33.1</v>
       </c>
       <c r="C34" t="n">
-        <v>0</v>
+        <v>33.53024531804003</v>
       </c>
       <c r="D34" t="n">
-        <v>-33.1</v>
+        <v>0.4302453180400292</v>
       </c>
       <c r="E34" t="n">
-        <v>1095.61</v>
+        <v>0.1851110336953659</v>
       </c>
     </row>
     <row r="35">
@@ -1024,13 +1024,13 @@
         <v>33.4</v>
       </c>
       <c r="C35" t="n">
-        <v>0</v>
+        <v>32.84650728479531</v>
       </c>
       <c r="D35" t="n">
-        <v>-33.4</v>
+        <v>-0.5534927152046905</v>
       </c>
       <c r="E35" t="n">
-        <v>1115.56</v>
+        <v>0.3063541857846606</v>
       </c>
     </row>
     <row r="36">
@@ -1041,13 +1041,13 @@
         <v>33.7</v>
       </c>
       <c r="C36" t="n">
-        <v>0</v>
+        <v>34.00686701367583</v>
       </c>
       <c r="D36" t="n">
-        <v>-33.7</v>
+        <v>0.3068670136758271</v>
       </c>
       <c r="E36" t="n">
-        <v>1135.69</v>
+        <v>0.09416736408232028</v>
       </c>
     </row>
     <row r="37">
@@ -1058,13 +1058,13 @@
         <v>34.1</v>
       </c>
       <c r="C37" t="n">
-        <v>0</v>
+        <v>34.89016021427642</v>
       </c>
       <c r="D37" t="n">
-        <v>-34.1</v>
+        <v>0.790160214276419</v>
       </c>
       <c r="E37" t="n">
-        <v>1162.81</v>
+        <v>0.6243531642253565</v>
       </c>
     </row>
     <row r="38">
@@ -1075,13 +1075,13 @@
         <v>34.4</v>
       </c>
       <c r="C38" t="n">
-        <v>0</v>
+        <v>35.13709982289468</v>
       </c>
       <c r="D38" t="n">
-        <v>-34.4</v>
+        <v>0.7370998228946846</v>
       </c>
       <c r="E38" t="n">
-        <v>1183.36</v>
+        <v>0.5433161489113754</v>
       </c>
     </row>
     <row r="39">
@@ -1092,13 +1092,13 @@
         <v>34.9</v>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>35.28494508555107</v>
       </c>
       <c r="D39" t="n">
-        <v>-34.9</v>
+        <v>0.3849450855510739</v>
       </c>
       <c r="E39" t="n">
-        <v>1218.01</v>
+        <v>0.1481827188899236</v>
       </c>
     </row>
     <row r="40">
@@ -1109,13 +1109,13 @@
         <v>35.3</v>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>34.84355280154394</v>
       </c>
       <c r="D40" t="n">
-        <v>-35.3</v>
+        <v>-0.4564471984560612</v>
       </c>
       <c r="E40" t="n">
-        <v>1246.09</v>
+        <v>0.2083440449783869</v>
       </c>
     </row>
     <row r="41">
@@ -1126,13 +1126,13 @@
         <v>35.7</v>
       </c>
       <c r="C41" t="n">
-        <v>0</v>
+        <v>35.66862906993612</v>
       </c>
       <c r="D41" t="n">
-        <v>-35.7</v>
+        <v>-0.03137093006388625</v>
       </c>
       <c r="E41" t="n">
-        <v>1274.49</v>
+        <v>0.0009841352530732422</v>
       </c>
     </row>
     <row r="42">
@@ -1143,13 +1143,13 @@
         <v>36.3</v>
       </c>
       <c r="C42" t="n">
-        <v>0</v>
+        <v>35.85962750787648</v>
       </c>
       <c r="D42" t="n">
-        <v>-36.3</v>
+        <v>-0.4403724921235153</v>
       </c>
       <c r="E42" t="n">
-        <v>1317.69</v>
+        <v>0.1939279318190755</v>
       </c>
     </row>
     <row r="43">
@@ -1160,13 +1160,13 @@
         <v>36.8</v>
       </c>
       <c r="C43" t="n">
-        <v>0</v>
+        <v>36.58988521355371</v>
       </c>
       <c r="D43" t="n">
-        <v>-36.8</v>
+        <v>-0.2101147864462831</v>
       </c>
       <c r="E43" t="n">
-        <v>1354.24</v>
+        <v>0.04414822348336716</v>
       </c>
     </row>
     <row r="44">
@@ -1177,13 +1177,13 @@
         <v>37.3</v>
       </c>
       <c r="C44" t="n">
-        <v>0</v>
+        <v>37.83083254539498</v>
       </c>
       <c r="D44" t="n">
-        <v>-37.3</v>
+        <v>0.5308325453949863</v>
       </c>
       <c r="E44" t="n">
-        <v>1391.29</v>
+        <v>0.2817831912505201</v>
       </c>
     </row>
     <row r="45">
@@ -1194,13 +1194,13 @@
         <v>37.9</v>
       </c>
       <c r="C45" t="n">
-        <v>0</v>
+        <v>39.01314395352769</v>
       </c>
       <c r="D45" t="n">
-        <v>-37.9</v>
+        <v>1.11314395352769</v>
       </c>
       <c r="E45" t="n">
-        <v>1436.41</v>
+        <v>1.239089461275255</v>
       </c>
     </row>
     <row r="46">
@@ -1211,13 +1211,13 @@
         <v>38.5</v>
       </c>
       <c r="C46" t="n">
-        <v>0</v>
+        <v>39.25621049148977</v>
       </c>
       <c r="D46" t="n">
-        <v>-38.5</v>
+        <v>0.7562104914897674</v>
       </c>
       <c r="E46" t="n">
-        <v>1482.25</v>
+        <v>0.5718543074391955</v>
       </c>
     </row>
     <row r="47">
@@ -1228,13 +1228,13 @@
         <v>38.9</v>
       </c>
       <c r="C47" t="n">
-        <v>0</v>
+        <v>39.2911214137161</v>
       </c>
       <c r="D47" t="n">
-        <v>-38.9</v>
+        <v>0.3911214137160997</v>
       </c>
       <c r="E47" t="n">
-        <v>1513.21</v>
+        <v>0.1529759602672804</v>
       </c>
     </row>
     <row r="48">
@@ -1245,13 +1245,13 @@
         <v>39.4</v>
       </c>
       <c r="C48" t="n">
-        <v>0</v>
+        <v>40.10510052842852</v>
       </c>
       <c r="D48" t="n">
-        <v>-39.4</v>
+        <v>0.7051005284285239</v>
       </c>
       <c r="E48" t="n">
-        <v>1552.36</v>
+        <v>0.4971667551901836</v>
       </c>
     </row>
     <row r="49">
@@ -1262,13 +1262,13 @@
         <v>39.9</v>
       </c>
       <c r="C49" t="n">
-        <v>0</v>
+        <v>39.87448722716134</v>
       </c>
       <c r="D49" t="n">
-        <v>-39.9</v>
+        <v>-0.02551277283865971</v>
       </c>
       <c r="E49" t="n">
-        <v>1592.01</v>
+        <v>0.0006509015779170528</v>
       </c>
     </row>
     <row r="50">
@@ -1279,13 +1279,13 @@
         <v>40.1</v>
       </c>
       <c r="C50" t="n">
-        <v>0</v>
+        <v>36.32202583591969</v>
       </c>
       <c r="D50" t="n">
-        <v>-40.1</v>
+        <v>-3.777974164080312</v>
       </c>
       <c r="E50" t="n">
-        <v>1608.01</v>
+        <v>14.27308878445833</v>
       </c>
     </row>
     <row r="51">
@@ -1296,13 +1296,13 @@
         <v>40.6</v>
       </c>
       <c r="C51" t="n">
-        <v>0</v>
+        <v>39.63872335809702</v>
       </c>
       <c r="D51" t="n">
-        <v>-40.6</v>
+        <v>-0.9612766419029768</v>
       </c>
       <c r="E51" t="n">
-        <v>1648.36</v>
+        <v>0.9240527822682639</v>
       </c>
     </row>
     <row r="52">
@@ -1313,11 +1313,11 @@
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="n">
-        <v>-1641.03</v>
+        <v>8.072418978433124</v>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="n">
-        <v>54420.1889</v>
+        <v>30.08121531779148</v>
       </c>
     </row>
     <row r="53">
@@ -1330,7 +1330,7 @@
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="n">
-        <v>1088.403778</v>
+        <v>0.6016243063558295</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Put in one file
</commit_message>
<xml_diff>
--- a/full/sliding_window_results_window_1.xlsx
+++ b/full/sliding_window_results_window_1.xlsx
@@ -463,13 +463,13 @@
         <v>28.98</v>
       </c>
       <c r="C2" t="n">
-        <v>29.72175776911019</v>
+        <v>29.15091033271521</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7417577691101904</v>
+        <v>0.1709103327152057</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5502045880353266</v>
+        <v>0.02921034182882232</v>
       </c>
     </row>
     <row r="3">
@@ -480,13 +480,13 @@
         <v>29.15</v>
       </c>
       <c r="C3" t="n">
-        <v>30.02891384579398</v>
+        <v>28.67086921649891</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8789138457939778</v>
+        <v>-0.4791307835010841</v>
       </c>
       <c r="E3" t="n">
-        <v>0.7724895483283601</v>
+        <v>0.2295663076983627</v>
       </c>
     </row>
     <row r="4">
@@ -497,13 +497,13 @@
         <v>29.35</v>
       </c>
       <c r="C4" t="n">
-        <v>29.87532757460375</v>
+        <v>28.59359961512243</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5253275746037467</v>
+        <v>-0.7564003848775762</v>
       </c>
       <c r="E4" t="n">
-        <v>0.275969060639055</v>
+        <v>0.5721415422429454</v>
       </c>
     </row>
     <row r="5">
@@ -514,13 +514,13 @@
         <v>29.37</v>
       </c>
       <c r="C5" t="n">
-        <v>29.64943781981881</v>
+        <v>28.72728691195743</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2794378198188099</v>
+        <v>-0.6427130880425729</v>
       </c>
       <c r="E5" t="n">
-        <v>0.07808549514508965</v>
+        <v>0.41308011354122</v>
       </c>
     </row>
     <row r="6">
@@ -531,13 +531,13 @@
         <v>29.54</v>
       </c>
       <c r="C6" t="n">
-        <v>30.2197193266033</v>
+        <v>29.60143929179227</v>
       </c>
       <c r="D6" t="n">
-        <v>0.6797193266032977</v>
+        <v>0.0614392917922757</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4620183629580405</v>
+        <v>0.003774786575936396</v>
       </c>
     </row>
     <row r="7">
@@ -548,13 +548,13 @@
         <v>29.55</v>
       </c>
       <c r="C7" t="n">
-        <v>30.16524852836157</v>
+        <v>29.62371283792032</v>
       </c>
       <c r="D7" t="n">
-        <v>0.6152485283615654</v>
+        <v>0.07371283792031846</v>
       </c>
       <c r="E7" t="n">
-        <v>0.378530751651072</v>
+        <v>0.00543358247426714</v>
       </c>
     </row>
     <row r="8">
@@ -565,13 +565,13 @@
         <v>29.75</v>
       </c>
       <c r="C8" t="n">
-        <v>30.95421275670812</v>
+        <v>29.66637735726204</v>
       </c>
       <c r="D8" t="n">
-        <v>1.20421275670812</v>
+        <v>-0.08362264273796072</v>
       </c>
       <c r="E8" t="n">
-        <v>1.45012836341857</v>
+        <v>0.006992746378480614</v>
       </c>
     </row>
     <row r="9">
@@ -582,13 +582,13 @@
         <v>29.84</v>
       </c>
       <c r="C9" t="n">
-        <v>30.3238393500008</v>
+        <v>29.84270492297819</v>
       </c>
       <c r="D9" t="n">
-        <v>0.483839350000796</v>
+        <v>0.002704922978193025</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2341005166091928</v>
+        <v>7.316608317956625e-06</v>
       </c>
     </row>
     <row r="10">
@@ -599,13 +599,13 @@
         <v>29.81</v>
       </c>
       <c r="C10" t="n">
-        <v>29.46879379716013</v>
+        <v>29.97765992443873</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.3412062028398708</v>
+        <v>0.1676599244387269</v>
       </c>
       <c r="E10" t="n">
-        <v>0.116421672856403</v>
+        <v>0.02810985026279961</v>
       </c>
     </row>
     <row r="11">
@@ -616,13 +616,13 @@
         <v>29.92</v>
       </c>
       <c r="C11" t="n">
-        <v>30.68162427992516</v>
+        <v>29.90365423835424</v>
       </c>
       <c r="D11" t="n">
-        <v>0.761624279925158</v>
+        <v>-0.01634576164576274</v>
       </c>
       <c r="E11" t="n">
-        <v>0.5800715437715155</v>
+        <v>0.0002671839237800881</v>
       </c>
     </row>
     <row r="12">
@@ -633,13 +633,13 @@
         <v>29.98</v>
       </c>
       <c r="C12" t="n">
-        <v>30.02526259058906</v>
+        <v>30.05089126187233</v>
       </c>
       <c r="D12" t="n">
-        <v>0.04526259058906135</v>
+        <v>0.07089126187232608</v>
       </c>
       <c r="E12" t="n">
-        <v>0.002048702106832985</v>
+        <v>0.005025571009850714</v>
       </c>
     </row>
     <row r="13">
@@ -650,13 +650,13 @@
         <v>30.04</v>
       </c>
       <c r="C13" t="n">
-        <v>29.65885848788355</v>
+        <v>30.03760920210035</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.3811415121164501</v>
+        <v>-0.002390797899646913</v>
       </c>
       <c r="E13" t="n">
-        <v>0.1452688522584141</v>
+        <v>5.715914596956089e-06</v>
       </c>
     </row>
     <row r="14">
@@ -667,13 +667,13 @@
         <v>30.21</v>
       </c>
       <c r="C14" t="n">
-        <v>30.0738608790388</v>
+        <v>29.78761085942527</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.1361391209612037</v>
+        <v>-0.4223891405747331</v>
       </c>
       <c r="E14" t="n">
-        <v>0.01853386025608926</v>
+        <v>0.1784125860754616</v>
       </c>
     </row>
     <row r="15">
@@ -684,13 +684,13 @@
         <v>30.22</v>
       </c>
       <c r="C15" t="n">
-        <v>29.9260358867717</v>
+        <v>29.83198067123257</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.2939641132282951</v>
+        <v>-0.3880193287674274</v>
       </c>
       <c r="E15" t="n">
-        <v>0.08641489986609789</v>
+        <v>0.1505589994971249</v>
       </c>
     </row>
     <row r="16">
@@ -701,13 +701,13 @@
         <v>30.38</v>
       </c>
       <c r="C16" t="n">
-        <v>29.94177716779699</v>
+        <v>29.82809165447258</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.4382228322030066</v>
+        <v>-0.5519083455274156</v>
       </c>
       <c r="E16" t="n">
-        <v>0.1920392506640245</v>
+        <v>0.3046028218628092</v>
       </c>
     </row>
     <row r="17">
@@ -718,13 +718,13 @@
         <v>30.44</v>
       </c>
       <c r="C17" t="n">
-        <v>29.90366860471718</v>
+        <v>29.93473684471761</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.5363313952828221</v>
+        <v>-0.5052631552823925</v>
       </c>
       <c r="E17" t="n">
-        <v>0.2876513655660188</v>
+        <v>0.2552908560859191</v>
       </c>
     </row>
     <row r="18">
@@ -735,13 +735,13 @@
         <v>30.48</v>
       </c>
       <c r="C18" t="n">
-        <v>29.86792644700605</v>
+        <v>30.32235284911957</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.6120735529939552</v>
+        <v>-0.1576471508804289</v>
       </c>
       <c r="E18" t="n">
-        <v>0.374634034274644</v>
+        <v>0.02485262418071672</v>
       </c>
     </row>
     <row r="19">
@@ -752,13 +752,13 @@
         <v>30.69</v>
       </c>
       <c r="C19" t="n">
-        <v>30.78666544642995</v>
+        <v>30.61478676844679</v>
       </c>
       <c r="D19" t="n">
-        <v>0.09666544642994523</v>
+        <v>-0.07521323155321369</v>
       </c>
       <c r="E19" t="n">
-        <v>0.009344208533500611</v>
+        <v>0.005657030200677339</v>
       </c>
     </row>
     <row r="20">
@@ -769,13 +769,13 @@
         <v>30.75</v>
       </c>
       <c r="C20" t="n">
-        <v>30.99431524769091</v>
+        <v>30.19549987913008</v>
       </c>
       <c r="D20" t="n">
-        <v>0.2443152476909134</v>
+        <v>-0.5545001208699212</v>
       </c>
       <c r="E20" t="n">
-        <v>0.05968994025427236</v>
+        <v>0.3074703840447572</v>
       </c>
     </row>
     <row r="21">
@@ -786,13 +786,13 @@
         <v>30.94</v>
       </c>
       <c r="C21" t="n">
-        <v>31.60933116519394</v>
+        <v>30.80147819617812</v>
       </c>
       <c r="D21" t="n">
-        <v>0.6693311651939347</v>
+        <v>-0.138521803821881</v>
       </c>
       <c r="E21" t="n">
-        <v>0.4480042086998702</v>
+        <v>0.01918829013406767</v>
       </c>
     </row>
     <row r="22">
@@ -803,13 +803,13 @@
         <v>30.95</v>
       </c>
       <c r="C22" t="n">
-        <v>31.35647702173609</v>
+        <v>30.83279632924468</v>
       </c>
       <c r="D22" t="n">
-        <v>0.4064770217360909</v>
+        <v>-0.1172036707553232</v>
       </c>
       <c r="E22" t="n">
-        <v>0.1652235691994425</v>
+        <v>0.01373670043852221</v>
       </c>
     </row>
     <row r="23">
@@ -820,13 +820,13 @@
         <v>31.02</v>
       </c>
       <c r="C23" t="n">
-        <v>31.14129646547685</v>
+        <v>31.04501157985084</v>
       </c>
       <c r="D23" t="n">
-        <v>0.1212964654768527</v>
+        <v>0.02501157985084035</v>
       </c>
       <c r="E23" t="n">
-        <v>0.01471283253717732</v>
+        <v>0.000625579126634963</v>
       </c>
     </row>
     <row r="24">
@@ -837,13 +837,13 @@
         <v>31.12</v>
       </c>
       <c r="C24" t="n">
-        <v>31.11198262567547</v>
+        <v>31.24246548021354</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.008017374324534643</v>
+        <v>0.1224654802135419</v>
       </c>
       <c r="E24" t="n">
-        <v>6.427829105970732e-05</v>
+        <v>0.01499779384393342</v>
       </c>
     </row>
     <row r="25">
@@ -854,13 +854,13 @@
         <v>31.28</v>
       </c>
       <c r="C25" t="n">
-        <v>31.61760285234385</v>
+        <v>31.51907741983583</v>
       </c>
       <c r="D25" t="n">
-        <v>0.3376028523438528</v>
+        <v>0.2390774198358336</v>
       </c>
       <c r="E25" t="n">
-        <v>0.1139756859107053</v>
+        <v>0.05715801267535946</v>
       </c>
     </row>
     <row r="26">
@@ -871,13 +871,13 @@
         <v>31.38</v>
       </c>
       <c r="C26" t="n">
-        <v>31.5746255466973</v>
+        <v>31.74824750231911</v>
       </c>
       <c r="D26" t="n">
-        <v>0.1946255466973028</v>
+        <v>0.3682475023191145</v>
       </c>
       <c r="E26" t="n">
-        <v>0.037879103427224</v>
+        <v>0.1356062229642662</v>
       </c>
     </row>
     <row r="27">
@@ -888,13 +888,13 @@
         <v>31.58</v>
       </c>
       <c r="C27" t="n">
-        <v>31.46276909702048</v>
+        <v>31.89156668208879</v>
       </c>
       <c r="D27" t="n">
-        <v>-0.117230902979518</v>
+        <v>0.3115666820887952</v>
       </c>
       <c r="E27" t="n">
-        <v>0.01374308461339316</v>
+        <v>0.09707379738782039</v>
       </c>
     </row>
     <row r="28">
@@ -905,13 +905,13 @@
         <v>31.65</v>
       </c>
       <c r="C28" t="n">
-        <v>31.6124046137601</v>
+        <v>31.59508561508043</v>
       </c>
       <c r="D28" t="n">
-        <v>-0.03759538623989656</v>
+        <v>-0.05491438491956657</v>
       </c>
       <c r="E28" t="n">
-        <v>0.001413413066527003</v>
+        <v>0.003015589671094321</v>
       </c>
     </row>
     <row r="29">
@@ -922,13 +922,13 @@
         <v>31.88</v>
       </c>
       <c r="C29" t="n">
-        <v>32.07227687734462</v>
+        <v>31.71291842438952</v>
       </c>
       <c r="D29" t="n">
-        <v>0.1922768773446215</v>
+        <v>-0.1670815756104744</v>
       </c>
       <c r="E29" t="n">
-        <v>0.03697039756139862</v>
+        <v>0.02791625290847868</v>
       </c>
     </row>
     <row r="30">
@@ -939,13 +939,13 @@
         <v>32.28</v>
       </c>
       <c r="C30" t="n">
-        <v>32.43597484441806</v>
+        <v>31.98873136312886</v>
       </c>
       <c r="D30" t="n">
-        <v>0.1559748444180542</v>
+        <v>-0.2912686368711412</v>
       </c>
       <c r="E30" t="n">
-        <v>0.02432815209123622</v>
+        <v>0.08483741882477273</v>
       </c>
     </row>
     <row r="31">
@@ -956,13 +956,13 @@
         <v>32.45</v>
       </c>
       <c r="C31" t="n">
-        <v>32.75777595936748</v>
+        <v>32.03820438205644</v>
       </c>
       <c r="D31" t="n">
-        <v>0.3077759593674756</v>
+        <v>-0.4117956179435609</v>
       </c>
       <c r="E31" t="n">
-        <v>0.09472604116456999</v>
+        <v>0.1695756309575192</v>
       </c>
     </row>
     <row r="32">
@@ -973,13 +973,13 @@
         <v>32.85</v>
       </c>
       <c r="C32" t="n">
-        <v>34.12422113804068</v>
+        <v>33.10931692410176</v>
       </c>
       <c r="D32" t="n">
-        <v>1.27422113804068</v>
+        <v>0.2593169241017605</v>
       </c>
       <c r="E32" t="n">
-        <v>1.623639508629686</v>
+        <v>0.06724526712559824</v>
       </c>
     </row>
     <row r="33">
@@ -990,13 +990,13 @@
         <v>32.9</v>
       </c>
       <c r="C33" t="n">
-        <v>33.96927027946951</v>
+        <v>32.78695910810221</v>
       </c>
       <c r="D33" t="n">
-        <v>1.069270279469514</v>
+        <v>-0.1130408918977892</v>
       </c>
       <c r="E33" t="n">
-        <v>1.143338930556812</v>
+        <v>0.01277824324104767</v>
       </c>
     </row>
     <row r="34">
@@ -1007,13 +1007,13 @@
         <v>33.1</v>
       </c>
       <c r="C34" t="n">
-        <v>33.53024531804003</v>
+        <v>33.15880749708899</v>
       </c>
       <c r="D34" t="n">
-        <v>0.4302453180400292</v>
+        <v>0.05880749708898492</v>
       </c>
       <c r="E34" t="n">
-        <v>0.1851110336953659</v>
+        <v>0.00345832171387097</v>
       </c>
     </row>
     <row r="35">
@@ -1024,13 +1024,13 @@
         <v>33.4</v>
       </c>
       <c r="C35" t="n">
-        <v>32.84650728479531</v>
+        <v>33.11086140922448</v>
       </c>
       <c r="D35" t="n">
-        <v>-0.5534927152046905</v>
+        <v>-0.2891385907755151</v>
       </c>
       <c r="E35" t="n">
-        <v>0.3063541857846606</v>
+        <v>0.08360112467565077</v>
       </c>
     </row>
     <row r="36">
@@ -1041,13 +1041,13 @@
         <v>33.7</v>
       </c>
       <c r="C36" t="n">
-        <v>34.00686701367583</v>
+        <v>33.72138313898149</v>
       </c>
       <c r="D36" t="n">
-        <v>0.3068670136758271</v>
+        <v>0.02138313898149136</v>
       </c>
       <c r="E36" t="n">
-        <v>0.09416736408232028</v>
+        <v>0.0004572386327017752</v>
       </c>
     </row>
     <row r="37">
@@ -1058,13 +1058,13 @@
         <v>34.1</v>
       </c>
       <c r="C37" t="n">
-        <v>34.89016021427642</v>
+        <v>34.44377180591287</v>
       </c>
       <c r="D37" t="n">
-        <v>0.790160214276419</v>
+        <v>0.3437718059128656</v>
       </c>
       <c r="E37" t="n">
-        <v>0.6243531642253565</v>
+        <v>0.1181790545405929</v>
       </c>
     </row>
     <row r="38">
@@ -1075,13 +1075,13 @@
         <v>34.4</v>
       </c>
       <c r="C38" t="n">
-        <v>35.13709982289468</v>
+        <v>34.50243634189844</v>
       </c>
       <c r="D38" t="n">
-        <v>0.7370998228946846</v>
+        <v>0.1024363418984393</v>
       </c>
       <c r="E38" t="n">
-        <v>0.5433161489113754</v>
+        <v>0.01049320414153395</v>
       </c>
     </row>
     <row r="39">
@@ -1092,13 +1092,13 @@
         <v>34.9</v>
       </c>
       <c r="C39" t="n">
-        <v>35.28494508555107</v>
+        <v>34.96445461375627</v>
       </c>
       <c r="D39" t="n">
-        <v>0.3849450855510739</v>
+        <v>0.06445461375627559</v>
       </c>
       <c r="E39" t="n">
-        <v>0.1481827188899236</v>
+        <v>0.004154397234470671</v>
       </c>
     </row>
     <row r="40">
@@ -1109,13 +1109,13 @@
         <v>35.3</v>
       </c>
       <c r="C40" t="n">
-        <v>34.84355280154394</v>
+        <v>34.64730527918477</v>
       </c>
       <c r="D40" t="n">
-        <v>-0.4564471984560612</v>
+        <v>-0.6526947208152265</v>
       </c>
       <c r="E40" t="n">
-        <v>0.2083440449783869</v>
+        <v>0.4260103985800665</v>
       </c>
     </row>
     <row r="41">
@@ -1126,13 +1126,13 @@
         <v>35.7</v>
       </c>
       <c r="C41" t="n">
-        <v>35.66862906993612</v>
+        <v>35.11439675203884</v>
       </c>
       <c r="D41" t="n">
-        <v>-0.03137093006388625</v>
+        <v>-0.5856032479611599</v>
       </c>
       <c r="E41" t="n">
-        <v>0.0009841352530732422</v>
+        <v>0.3429311640226598</v>
       </c>
     </row>
     <row r="42">
@@ -1143,13 +1143,13 @@
         <v>36.3</v>
       </c>
       <c r="C42" t="n">
-        <v>35.85962750787648</v>
+        <v>36.00216725834134</v>
       </c>
       <c r="D42" t="n">
-        <v>-0.4403724921235153</v>
+        <v>-0.2978327416586595</v>
       </c>
       <c r="E42" t="n">
-        <v>0.1939279318190755</v>
+        <v>0.08870434200391379</v>
       </c>
     </row>
     <row r="43">
@@ -1160,13 +1160,13 @@
         <v>36.8</v>
       </c>
       <c r="C43" t="n">
-        <v>36.58988521355371</v>
+        <v>36.37442724091371</v>
       </c>
       <c r="D43" t="n">
-        <v>-0.2101147864462831</v>
+        <v>-0.4255727590862861</v>
       </c>
       <c r="E43" t="n">
-        <v>0.04414822348336716</v>
+        <v>0.1811121732763141</v>
       </c>
     </row>
     <row r="44">
@@ -1177,13 +1177,13 @@
         <v>37.3</v>
       </c>
       <c r="C44" t="n">
-        <v>37.83083254539498</v>
+        <v>37.38406080059678</v>
       </c>
       <c r="D44" t="n">
-        <v>0.5308325453949863</v>
+        <v>0.08406080059678089</v>
       </c>
       <c r="E44" t="n">
-        <v>0.2817831912505201</v>
+        <v>0.007066218196971759</v>
       </c>
     </row>
     <row r="45">
@@ -1194,13 +1194,13 @@
         <v>37.9</v>
       </c>
       <c r="C45" t="n">
-        <v>39.01314395352769</v>
+        <v>37.94210030973155</v>
       </c>
       <c r="D45" t="n">
-        <v>1.11314395352769</v>
+        <v>0.04210030973155199</v>
       </c>
       <c r="E45" t="n">
-        <v>1.239089461275255</v>
+        <v>0.001772436079492611</v>
       </c>
     </row>
     <row r="46">
@@ -1211,13 +1211,13 @@
         <v>38.5</v>
       </c>
       <c r="C46" t="n">
-        <v>39.25621049148977</v>
+        <v>38.29955586414763</v>
       </c>
       <c r="D46" t="n">
-        <v>0.7562104914897674</v>
+        <v>-0.2004441358523721</v>
       </c>
       <c r="E46" t="n">
-        <v>0.5718543074391955</v>
+        <v>0.0401778515976042</v>
       </c>
     </row>
     <row r="47">
@@ -1228,13 +1228,13 @@
         <v>38.9</v>
       </c>
       <c r="C47" t="n">
-        <v>39.2911214137161</v>
+        <v>38.81064811979377</v>
       </c>
       <c r="D47" t="n">
-        <v>0.3911214137160997</v>
+        <v>-0.08935188020623031</v>
       </c>
       <c r="E47" t="n">
-        <v>0.1529759602672804</v>
+        <v>0.007983758496388531</v>
       </c>
     </row>
     <row r="48">
@@ -1245,13 +1245,13 @@
         <v>39.4</v>
       </c>
       <c r="C48" t="n">
-        <v>40.10510052842852</v>
+        <v>39.32351519886852</v>
       </c>
       <c r="D48" t="n">
-        <v>0.7051005284285239</v>
+        <v>-0.07648480113147826</v>
       </c>
       <c r="E48" t="n">
-        <v>0.4971667551901836</v>
+        <v>0.005849924804121779</v>
       </c>
     </row>
     <row r="49">
@@ -1262,13 +1262,13 @@
         <v>39.9</v>
       </c>
       <c r="C49" t="n">
-        <v>39.87448722716134</v>
+        <v>39.74260215855035</v>
       </c>
       <c r="D49" t="n">
-        <v>-0.02551277283865971</v>
+        <v>-0.1573978414496437</v>
       </c>
       <c r="E49" t="n">
-        <v>0.0006509015779170528</v>
+        <v>0.02477408049300719</v>
       </c>
     </row>
     <row r="50">
@@ -1279,13 +1279,13 @@
         <v>40.1</v>
       </c>
       <c r="C50" t="n">
-        <v>36.32202583591969</v>
+        <v>39.71392340055714</v>
       </c>
       <c r="D50" t="n">
-        <v>-3.777974164080312</v>
+        <v>-0.386076599442859</v>
       </c>
       <c r="E50" t="n">
-        <v>14.27308878445833</v>
+        <v>0.1490551406373618</v>
       </c>
     </row>
     <row r="51">
@@ -1296,13 +1296,13 @@
         <v>40.6</v>
       </c>
       <c r="C51" t="n">
-        <v>39.63872335809702</v>
+        <v>40.3692112874656</v>
       </c>
       <c r="D51" t="n">
-        <v>-0.9612766419029768</v>
+        <v>-0.2307887125344052</v>
       </c>
       <c r="E51" t="n">
-        <v>0.9240527822682639</v>
+        <v>0.05326342983328834</v>
       </c>
     </row>
     <row r="52">
@@ -1313,11 +1313,11 @@
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="n">
-        <v>8.072418978433124</v>
+        <v>-6.730737876800386</v>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="n">
-        <v>30.08121531779148</v>
+        <v>4.773259418665972</v>
       </c>
     </row>
     <row r="53">
@@ -1330,7 +1330,7 @@
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="n">
-        <v>0.6016243063558295</v>
+        <v>0.09546518837331945</v>
       </c>
     </row>
   </sheetData>

</xml_diff>